<commit_message>
feat(db): capa de acceso a DB PostgreSQL - entidades Vehicle+ImportLog, repositorios con cleanup/polling/queries
</commit_message>
<xml_diff>
--- a/Automated-Testing/data/Vehicle-To-Import.xlsx
+++ b/Automated-Testing/data/Vehicle-To-Import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jhon Martinez\Documents\Motorambar\QA-Motorambar-2.0\Automated-Testing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA036940-D032-4768-81BB-BA883F62C3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B47CF57-AD47-4CE7-8A5A-46047403CCED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="162">
   <si>
     <t>VIN</t>
   </si>
@@ -427,24 +427,6 @@
     <t>BANCO POPULAR</t>
   </si>
   <si>
-    <t>MEDINA KIA</t>
-  </si>
-  <si>
-    <t>MARCA AUTOMOTIVE DEL NORTE LLC</t>
-  </si>
-  <si>
-    <t>ADRIEL KIA</t>
-  </si>
-  <si>
-    <t>AGUADILLA AUTO CENTER, INC.</t>
-  </si>
-  <si>
-    <t>AUTOMAS DEL CARIBE LLC</t>
-  </si>
-  <si>
-    <t>AUTO STOP SAN SEBASTIAN, INC.</t>
-  </si>
-  <si>
     <t>PEPE ABAD NISSAN</t>
   </si>
   <si>
@@ -491,6 +473,39 @@
   </si>
   <si>
     <t>RED</t>
+  </si>
+  <si>
+    <t>MEDINA NISSAN</t>
+  </si>
+  <si>
+    <t>YOKOMURO NISSAN</t>
+  </si>
+  <si>
+    <t>C1105</t>
+  </si>
+  <si>
+    <t>C1108</t>
+  </si>
+  <si>
+    <t>100000042</t>
+  </si>
+  <si>
+    <t>100002574</t>
+  </si>
+  <si>
+    <t>100000024</t>
+  </si>
+  <si>
+    <t>100000074</t>
+  </si>
+  <si>
+    <t>100000027</t>
+  </si>
+  <si>
+    <t>100000022</t>
+  </si>
+  <si>
+    <t>100000049</t>
   </si>
 </sst>
 </file>
@@ -548,7 +563,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -565,69 +580,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1143,7 +1095,7 @@
         <v>101</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C2" s="2">
         <v>187</v>
@@ -1193,8 +1145,8 @@
       <c r="R2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S2" s="25" t="s">
-        <v>135</v>
+      <c r="S2" s="6" t="s">
+        <v>102</v>
       </c>
       <c r="T2" s="2" t="s">
         <v>46</v>
@@ -1208,7 +1160,7 @@
       <c r="W2" s="2">
         <v>8889</v>
       </c>
-      <c r="X2" s="22" t="s">
+      <c r="X2" s="2" t="s">
         <v>129</v>
       </c>
       <c r="Y2" s="2" t="s">
@@ -1223,10 +1175,10 @@
       <c r="AB2" s="2">
         <v>660763584</v>
       </c>
-      <c r="AC2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD2" s="6" t="s">
+      <c r="AC2" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="AD2" s="2" t="s">
         <v>102</v>
       </c>
       <c r="AE2" s="2" t="s">
@@ -1265,7 +1217,7 @@
         <v>46177</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F3" s="4">
         <v>32145.5</v>
@@ -1277,7 +1229,7 @@
         <v>46190</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>40</v>
@@ -1306,8 +1258,8 @@
       <c r="R3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S3" s="26" t="s">
-        <v>136</v>
+      <c r="S3" s="7" t="s">
+        <v>103</v>
       </c>
       <c r="T3" s="2" t="s">
         <v>56</v>
@@ -1336,19 +1288,19 @@
       <c r="AB3" s="2">
         <v>661845927</v>
       </c>
-      <c r="AC3" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD3" s="7" t="s">
+      <c r="AC3" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="AD3" s="2" t="s">
         <v>103</v>
       </c>
       <c r="AE3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="AF3" s="21" t="s">
+      <c r="AF3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="AG3" s="21" t="s">
+      <c r="AG3" s="2" t="s">
         <v>112</v>
       </c>
       <c r="AH3" s="2" t="s">
@@ -1366,7 +1318,7 @@
         <v>92</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C4" s="2">
         <v>191</v>
@@ -1375,7 +1327,7 @@
         <v>46178</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F4" s="4">
         <v>33698.25</v>
@@ -1387,7 +1339,7 @@
         <v>46191</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>40</v>
@@ -1416,8 +1368,8 @@
       <c r="R4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S4" s="27" t="s">
-        <v>137</v>
+      <c r="S4" s="8" t="s">
+        <v>151</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>60</v>
@@ -1431,7 +1383,7 @@
       <c r="W4" s="2">
         <v>8889</v>
       </c>
-      <c r="X4" s="23" t="s">
+      <c r="X4" s="2" t="s">
         <v>130</v>
       </c>
       <c r="Y4" s="2" t="s">
@@ -1446,10 +1398,10 @@
       <c r="AB4" s="2">
         <v>663102418</v>
       </c>
-      <c r="AC4" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD4" s="8" t="s">
+      <c r="AC4" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="AD4" s="2" t="s">
         <v>104</v>
       </c>
       <c r="AE4" s="2" t="s">
@@ -1458,7 +1410,7 @@
       <c r="AF4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG4" s="21" t="s">
+      <c r="AG4" s="2" t="s">
         <v>115</v>
       </c>
       <c r="AH4" s="2" t="s">
@@ -1479,7 +1431,7 @@
         <v>93</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C5" s="2">
         <v>147</v>
@@ -1488,7 +1440,7 @@
         <v>46179</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F5" s="4">
         <v>35214.9</v>
@@ -1500,7 +1452,7 @@
         <v>46192</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>40</v>
@@ -1529,7 +1481,7 @@
       <c r="R5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S5" s="28" t="s">
+      <c r="S5" s="2" t="s">
         <v>110</v>
       </c>
       <c r="T5" s="2" t="s">
@@ -1544,7 +1496,7 @@
       <c r="W5" s="2">
         <v>7778</v>
       </c>
-      <c r="X5" s="24" t="s">
+      <c r="X5" s="2" t="s">
         <v>131</v>
       </c>
       <c r="Y5" s="2" t="s">
@@ -1559,10 +1511,10 @@
       <c r="AB5" s="2">
         <v>664578391</v>
       </c>
-      <c r="AC5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD5" s="9" t="s">
+      <c r="AC5" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="AD5" s="2" t="s">
         <v>105</v>
       </c>
       <c r="AE5" s="2" t="s">
@@ -1571,7 +1523,7 @@
       <c r="AF5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG5" s="21" t="s">
+      <c r="AG5" s="2" t="s">
         <v>115</v>
       </c>
       <c r="AH5" s="2" t="s">
@@ -1601,7 +1553,7 @@
         <v>46180</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F6" s="4">
         <v>36857.4</v>
@@ -1613,7 +1565,7 @@
         <v>46193</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>40</v>
@@ -1642,8 +1594,8 @@
       <c r="R6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S6" s="29" t="s">
-        <v>136</v>
+      <c r="S6" s="9" t="s">
+        <v>105</v>
       </c>
       <c r="T6" s="2" t="s">
         <v>68</v>
@@ -1672,10 +1624,10 @@
       <c r="AB6" s="2">
         <v>665914206</v>
       </c>
-      <c r="AC6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD6" s="10" t="s">
+      <c r="AC6" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD6" s="2" t="s">
         <v>106</v>
       </c>
       <c r="AE6" s="2" t="s">
@@ -1684,7 +1636,7 @@
       <c r="AF6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG6" s="20" t="s">
+      <c r="AG6" s="2" t="s">
         <v>116</v>
       </c>
       <c r="AH6" s="2" t="s">
@@ -1705,7 +1657,7 @@
         <v>95</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C7" s="2">
         <v>149</v>
@@ -1714,7 +1666,7 @@
         <v>46181</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F7" s="4">
         <v>38126.75</v>
@@ -1726,10 +1678,10 @@
         <v>46194</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K7" s="2">
         <v>2025</v>
@@ -1755,8 +1707,8 @@
       <c r="R7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S7" s="30" t="s">
-        <v>138</v>
+      <c r="S7" s="10" t="s">
+        <v>152</v>
       </c>
       <c r="T7" s="2" t="s">
         <v>72</v>
@@ -1785,10 +1737,10 @@
       <c r="AB7" s="2">
         <v>667281543</v>
       </c>
-      <c r="AC7" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD7" s="11" t="s">
+      <c r="AC7" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="AD7" s="2" t="s">
         <v>107</v>
       </c>
       <c r="AE7" s="2" t="s">
@@ -1797,7 +1749,7 @@
       <c r="AF7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG7" s="19" t="s">
+      <c r="AG7" s="2" t="s">
         <v>115</v>
       </c>
       <c r="AH7" s="2" t="s">
@@ -1818,7 +1770,7 @@
         <v>96</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C8" s="2">
         <v>188</v>
@@ -1827,7 +1779,7 @@
         <v>46182</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="F8" s="4">
         <v>39543.599999999999</v>
@@ -1839,10 +1791,10 @@
         <v>46195</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K8" s="2">
         <v>2024</v>
@@ -1868,8 +1820,8 @@
       <c r="R8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S8" s="31" t="s">
-        <v>139</v>
+      <c r="S8" s="11" t="s">
+        <v>109</v>
       </c>
       <c r="T8" s="2" t="s">
         <v>76</v>
@@ -1898,10 +1850,10 @@
       <c r="AB8" s="2">
         <v>668730195</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD8" s="13" t="s">
+      <c r="AC8" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="AD8" s="2" t="s">
         <v>109</v>
       </c>
       <c r="AE8" s="2" t="s">
@@ -1910,7 +1862,7 @@
       <c r="AF8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG8" s="18" t="s">
+      <c r="AG8" s="2" t="s">
         <v>114</v>
       </c>
       <c r="AH8" s="2" t="s">
@@ -1940,7 +1892,7 @@
         <v>46183</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F9" s="4">
         <v>41082.15</v>
@@ -1952,10 +1904,10 @@
         <v>46196</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K9" s="2">
         <v>2024</v>
@@ -1981,8 +1933,8 @@
       <c r="R9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S9" s="32" t="s">
-        <v>140</v>
+      <c r="S9" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="T9" s="2" t="s">
         <v>80</v>
@@ -2011,10 +1963,10 @@
       <c r="AB9" s="2">
         <v>669154872</v>
       </c>
-      <c r="AC9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD9" s="14" t="s">
+      <c r="AC9" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="AD9" s="2" t="s">
         <v>110</v>
       </c>
       <c r="AE9" s="2" t="s">
@@ -2023,7 +1975,7 @@
       <c r="AF9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG9" s="17" t="s">
+      <c r="AG9" s="2" t="s">
         <v>113</v>
       </c>
       <c r="AH9" s="2" t="s">
@@ -2044,7 +1996,7 @@
         <v>98</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C10" s="2">
         <v>201</v>
@@ -2065,10 +2017,10 @@
         <v>46197</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K10" s="2">
         <v>2024</v>
@@ -2094,8 +2046,8 @@
       <c r="R10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="S10" s="33" t="s">
-        <v>141</v>
+      <c r="S10" s="12" t="s">
+        <v>135</v>
       </c>
       <c r="T10" s="2" t="s">
         <v>84</v>
@@ -2124,10 +2076,10 @@
       <c r="AB10" s="2">
         <v>670842361</v>
       </c>
-      <c r="AC10" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD10" s="12" t="s">
+      <c r="AC10" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="AD10" s="2" t="s">
         <v>108</v>
       </c>
       <c r="AE10" s="2" t="s">
@@ -2136,7 +2088,7 @@
       <c r="AF10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG10" s="16" t="s">
+      <c r="AG10" s="2" t="s">
         <v>112</v>
       </c>
       <c r="AH10" s="2" t="s">
@@ -2157,7 +2109,7 @@
         <v>99</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2">
         <v>310</v>
@@ -2178,10 +2130,10 @@
         <v>46198</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K11" s="2">
         <v>2024</v>
@@ -2233,7 +2185,7 @@
       <c r="AB11" s="2">
         <v>672519804</v>
       </c>
-      <c r="AC11" s="2" t="s">
+      <c r="AC11" s="12" t="s">
         <v>50</v>
       </c>
       <c r="AD11" s="2" t="s">
@@ -2245,7 +2197,7 @@
       <c r="AF11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AG11" s="15" t="s">
+      <c r="AG11" s="2" t="s">
         <v>111</v>
       </c>
       <c r="AH11" s="2" t="s">
@@ -2267,6 +2219,7 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{92629465-E94C-48F9-A764-1784E4383F99}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>